<commit_message>
Separa OL da Aché (36 itens) dos pedidos de distribuidor
O controle não marca itens Aché na coluna OL; identifica-os pelo prefixo
GS1 7896658 nos EANs e gera OL_ACHE_04-09-2026.xlsx, removendo-os dos
pedidos ePan, SB LOG, Tapajós e Nazária e do comparativo.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VLivvbyTHZf5HaiMxTfGPo
</commit_message>
<xml_diff>
--- a/cotacoes/2026-09-04/PEDIDO_SBLOG_04-09-2026.xlsx
+++ b/cotacoes/2026-09-04/PEDIDO_SBLOG_04-09-2026.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1718,59 +1718,59 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>796541</t>
+          <t>11398</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>262941</v>
+        <v>431061</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>7896658036996</t>
+          <t>7898560661563</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>ALLESTRA 20 20+75MCG 63CPR</t>
+          <t>REPARIL GEL 30G</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>PV ALLESTRA 20/75MCG (CAIXA C/ 3 CARTELAS)</t>
+          <t>REPARIL 10+50MG/G GEL BG 30G</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>69.5</v>
+        <v>32.3</v>
       </c>
       <c r="J21" s="4">
         <f>G21*I21</f>
         <v/>
       </c>
       <c r="K21" s="4" t="n">
-        <v>69.5</v>
+        <v>32.3</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>22.18</v>
+        <v>32.3</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>22.18</v>
+        <v>27.27</v>
       </c>
       <c r="N21" s="5">
         <f>K21/L21-1</f>
         <v/>
       </c>
-      <c r="O21" s="6" t="inlineStr">
-        <is>
-          <t>ACIMA +213.3% (vs últ. compra)</t>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr"/>
@@ -1778,51 +1778,51 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>11398</t>
+          <t>761671</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>431061</v>
+        <v>444281</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>7898560661563</t>
+          <t>7896206402853</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>REPARIL GEL 30G</t>
+          <t>SELOZOK 25MG 30CPR</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>REPARIL 10+50MG/G GEL BG 30G</t>
+          <t>SELOZOK 25MG CX 30 COMP</t>
         </is>
       </c>
       <c r="F22" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>32.3</v>
+        <v>30</v>
       </c>
       <c r="J22" s="4">
         <f>G22*I22</f>
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>32.3</v>
+        <v>30</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>32.3</v>
+        <v>31.175</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>27.27</v>
+        <v>28.245</v>
       </c>
       <c r="N22" s="5">
         <f>K22/L22-1</f>
@@ -1838,25 +1838,25 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>761671</t>
+          <t>796508</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>444281</v>
+        <v>433961</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>7896206402853</t>
+          <t>7897460401750</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>SELOZOK 25MG 30CPR</t>
+          <t>SILIMALON 140+140+100MG 60CPR REV</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>SELOZOK 25MG CX 30 COMP</t>
+          <t>SILIMALON 140 140+100MG CX 60 COMP REV</t>
         </is>
       </c>
       <c r="F23" s="3" t="n">
@@ -1869,28 +1869,28 @@
         <v>1</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>30</v>
+        <v>148.3</v>
       </c>
       <c r="J23" s="4">
         <f>G23*I23</f>
         <v/>
       </c>
       <c r="K23" s="4" t="n">
-        <v>30</v>
+        <v>148.3</v>
       </c>
       <c r="L23" s="4" t="n">
-        <v>31.175</v>
+        <v>128.47</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>28.245</v>
+        <v>128.47</v>
       </c>
       <c r="N23" s="5">
         <f>K23/L23-1</f>
         <v/>
       </c>
-      <c r="O23" s="7" t="inlineStr">
-        <is>
-          <t>OK (≤ últ. compra)</t>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>ACIMA +15.4% (vs últ. compra)</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr"/>
@@ -1898,25 +1898,25 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>796508</t>
+          <t>700797</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>433961</v>
+        <v>297921</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>7897460401750</t>
+          <t>7898074617803</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>SILIMALON 140+140+100MG 60CPR REV</t>
+          <t>SPIDUFEN 600MG 10ENV 3G</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>SILIMALON 140 140+100MG CX 60 COMP REV</t>
+          <t>SPIDUFEN 1155MG GRAN SOL CX 10 ENV 3G SB DAMASCO</t>
         </is>
       </c>
       <c r="F24" s="3" t="n">
@@ -1929,28 +1929,28 @@
         <v>1</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>148.3</v>
+        <v>41.3</v>
       </c>
       <c r="J24" s="4">
         <f>G24*I24</f>
         <v/>
       </c>
       <c r="K24" s="4" t="n">
-        <v>148.3</v>
+        <v>41.3</v>
       </c>
       <c r="L24" s="4" t="n">
-        <v>128.47</v>
+        <v>42.05</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>128.47</v>
+        <v>36.49</v>
       </c>
       <c r="N24" s="5">
         <f>K24/L24-1</f>
         <v/>
       </c>
-      <c r="O24" s="6" t="inlineStr">
-        <is>
-          <t>ACIMA +15.4% (vs últ. compra)</t>
+      <c r="O24" s="7" t="inlineStr">
+        <is>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr"/>
@@ -1958,25 +1958,25 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>700797</t>
+          <t>775679</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>297921</v>
+        <v>455901</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>7898074617803</t>
+          <t>7896094206014</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>SPIDUFEN 600MG 10ENV 3G</t>
+          <t>TARFIC POM 0,3MG 10G</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>SPIDUFEN 1155MG GRAN SOL CX 10 ENV 3G SB DAMASCO</t>
+          <t>TARFIC 0,3MG POM BG 10G</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
@@ -1989,28 +1989,28 @@
         <v>1</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>41.3</v>
+        <v>76.7</v>
       </c>
       <c r="J25" s="4">
         <f>G25*I25</f>
         <v/>
       </c>
       <c r="K25" s="4" t="n">
-        <v>41.3</v>
+        <v>76.7</v>
       </c>
       <c r="L25" s="4" t="n">
-        <v>42.05</v>
+        <v>72.27</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>36.49</v>
+        <v>72.27</v>
       </c>
       <c r="N25" s="5">
         <f>K25/L25-1</f>
         <v/>
       </c>
-      <c r="O25" s="7" t="inlineStr">
-        <is>
-          <t>OK (≤ últ. compra)</t>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>ACIMA +6.1% (vs últ. compra)</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr"/>
@@ -2018,25 +2018,25 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>775679</t>
+          <t>775681</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>455901</v>
+        <v>455861</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>7896094206014</t>
+          <t>7896094206038</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>TARFIC POM 0,3MG 10G</t>
+          <t>TARFIC POM 1,0MG 10G</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>TARFIC 0,3MG POM BG 10G</t>
+          <t>TARFIC 1,0MG POM BG 10G</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
@@ -2049,20 +2049,20 @@
         <v>1</v>
       </c>
       <c r="I26" s="4" t="n">
-        <v>76.7</v>
+        <v>76.5</v>
       </c>
       <c r="J26" s="4">
         <f>G26*I26</f>
         <v/>
       </c>
       <c r="K26" s="4" t="n">
-        <v>76.7</v>
+        <v>76.5</v>
       </c>
       <c r="L26" s="4" t="n">
-        <v>72.27</v>
+        <v>72.27500000000001</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>72.27</v>
+        <v>72.27500000000001</v>
       </c>
       <c r="N26" s="5">
         <f>K26/L26-1</f>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
-          <t>ACIMA +6.1% (vs últ. compra)</t>
+          <t>ACIMA +5.8% (vs últ. compra)</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr"/>
@@ -2078,51 +2078,51 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>775681</t>
+          <t>771612</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>455861</v>
+        <v>395781</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>7896094206038</t>
+          <t>7891010986155</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>TARFIC POM 1,0MG 10G</t>
+          <t>TYLENOL 500MG 20CPR</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>TARFIC 1,0MG POM BG 10G</t>
+          <t>TYLENOL 500MG CX 20 COMP REV</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>76.5</v>
+        <v>29.8</v>
       </c>
       <c r="J27" s="4">
         <f>G27*I27</f>
         <v/>
       </c>
       <c r="K27" s="4" t="n">
-        <v>76.5</v>
+        <v>29.8</v>
       </c>
       <c r="L27" s="4" t="n">
-        <v>72.27500000000001</v>
+        <v>27.43</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>72.27500000000001</v>
+        <v>27.43</v>
       </c>
       <c r="N27" s="5">
         <f>K27/L27-1</f>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t>ACIMA +5.8% (vs últ. compra)</t>
+          <t>ACIMA +8.6% (vs últ. compra)</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr"/>
@@ -2138,51 +2138,51 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>771612</t>
+          <t>742106</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>395781</v>
+        <v>398541</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>7891010986155</t>
+          <t>7891010256968</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>TYLENOL 500MG 20CPR</t>
+          <t>TYLENOL SINUS 500MG+30MG 24CPR REV</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>TYLENOL 500MG CX 20 COMP REV</t>
+          <t>TYLENOL SINUS 500+30MG CX 24 COMP REV</t>
         </is>
       </c>
       <c r="F28" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>29.8</v>
+        <v>18.1</v>
       </c>
       <c r="J28" s="4">
         <f>G28*I28</f>
         <v/>
       </c>
       <c r="K28" s="4" t="n">
-        <v>29.8</v>
+        <v>18.1</v>
       </c>
       <c r="L28" s="4" t="n">
-        <v>27.43</v>
+        <v>16.83</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>27.43</v>
+        <v>16.8</v>
       </c>
       <c r="N28" s="5">
         <f>K28/L28-1</f>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
-          <t>ACIMA +8.6% (vs últ. compra)</t>
+          <t>ACIMA +7.5% (vs últ. compra)</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr"/>
@@ -2198,51 +2198,51 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>742106</t>
+          <t>794244</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>398541</v>
+        <v>344301</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>7891010256968</t>
+          <t>7896641808777</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>TYLENOL SINUS 500MG+30MG 24CPR REV</t>
+          <t>MESACOL 250MG 15SUP</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>TYLENOL SINUS 500+30MG CX 24 COMP REV</t>
+          <t>VENCIDO - PV MESACOL 250 MG SUP RET CT BERCO X 15</t>
         </is>
       </c>
       <c r="F29" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>18.1</v>
+        <v>60.6</v>
       </c>
       <c r="J29" s="4">
         <f>G29*I29</f>
         <v/>
       </c>
       <c r="K29" s="4" t="n">
-        <v>18.1</v>
+        <v>60.6</v>
       </c>
       <c r="L29" s="4" t="n">
-        <v>16.83</v>
+        <v>56.86</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>16.8</v>
+        <v>56.86</v>
       </c>
       <c r="N29" s="5">
         <f>K29/L29-1</f>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
-          <t>ACIMA +7.5% (vs últ. compra)</t>
+          <t>ACIMA +6.6% (vs últ. compra)</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2258,51 +2258,51 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>794244</t>
+          <t>799357</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>344301</v>
+        <v>610801</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>7896641808777</t>
+          <t>7500435209786</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>MESACOL 250MG 15SUP</t>
+          <t>VICK XPE MEL 100ML</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>VENCIDO - PV MESACOL 250 MG SUP RET CT BERCO X 15</t>
+          <t>VICK XAROPE XAROPE MIEL 100ML</t>
         </is>
       </c>
       <c r="F30" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I30" s="4" t="n">
-        <v>60.6</v>
+        <v>30</v>
       </c>
       <c r="J30" s="4">
         <f>G30*I30</f>
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>60.6</v>
+        <v>30</v>
       </c>
       <c r="L30" s="4" t="n">
-        <v>56.86</v>
+        <v>28.7366666666667</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>56.86</v>
+        <v>24.38</v>
       </c>
       <c r="N30" s="5">
         <f>K30/L30-1</f>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
-          <t>ACIMA +6.6% (vs últ. compra)</t>
+          <t>ACIMA +4.4% (vs últ. compra)</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr"/>
@@ -2318,51 +2318,51 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>799357</t>
+          <t>799472</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>610801</v>
+        <v>671911</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>7500435209786</t>
+          <t>7896004780818</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>VICK XPE MEL 100ML</t>
+          <t>VIOFTA 0,40% SOL OFTA 10ML</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>VICK XAROPE XAROPE MIEL 100ML</t>
+          <t>VIOFTA 0,40% SOL OFT 10ML-DEMAIS PROD</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>30</v>
+        <v>62.7</v>
       </c>
       <c r="J31" s="4">
         <f>G31*I31</f>
         <v/>
       </c>
       <c r="K31" s="4" t="n">
-        <v>30</v>
+        <v>62.7</v>
       </c>
       <c r="L31" s="4" t="n">
-        <v>28.7366666666667</v>
+        <v>53.03</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>24.38</v>
+        <v>53.03</v>
       </c>
       <c r="N31" s="5">
         <f>K31/L31-1</f>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
-          <t>ACIMA +4.4% (vs últ. compra)</t>
+          <t>ACIMA +18.2% (vs últ. compra)</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2378,51 +2378,51 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>799472</t>
+          <t>765174</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>671911</v>
+        <v>468541</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>7896004780818</t>
+          <t>7897129303579</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>VIOFTA 0,40% SOL OFTA 10ML</t>
+          <t>VITACID XT CR 1MG/G 25G</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>VIOFTA 0,40% SOL OFT 10ML-DEMAIS PROD</t>
+          <t>VITACID XT 1,00MG/G CREME DERM BG 25G</t>
         </is>
       </c>
       <c r="F32" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>62.7</v>
+        <v>58.7</v>
       </c>
       <c r="J32" s="4">
         <f>G32*I32</f>
         <v/>
       </c>
       <c r="K32" s="4" t="n">
-        <v>62.7</v>
+        <v>58.7</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>53.03</v>
+        <v>47.28</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>53.03</v>
+        <v>47.28</v>
       </c>
       <c r="N32" s="5">
         <f>K32/L32-1</f>
@@ -2430,7 +2430,7 @@
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
-          <t>ACIMA +18.2% (vs últ. compra)</t>
+          <t>ACIMA +24.2% (vs últ. compra)</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr"/>
@@ -2438,59 +2438,59 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>765174</t>
+          <t>718981</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>468541</v>
+        <v>65101</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>7897129303579</t>
+          <t>7590002023228</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>VITACID XT CR 1MG/G 25G</t>
+          <t>VICK XPE 44E 120ML</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>VITACID XT 1,00MG/G CREME DERM BG 25G</t>
+          <t>XAROPE 44 E 1,30+13,30MG/ML XPE FR 120ML</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I33" s="4" t="n">
-        <v>58.7</v>
+        <v>30</v>
       </c>
       <c r="J33" s="4">
         <f>G33*I33</f>
         <v/>
       </c>
       <c r="K33" s="4" t="n">
-        <v>58.7</v>
+        <v>30</v>
       </c>
       <c r="L33" s="4" t="n">
-        <v>47.28</v>
+        <v>30.73</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>47.28</v>
+        <v>23.2152</v>
       </c>
       <c r="N33" s="5">
         <f>K33/L33-1</f>
         <v/>
       </c>
-      <c r="O33" s="6" t="inlineStr">
-        <is>
-          <t>ACIMA +24.2% (vs últ. compra)</t>
+      <c r="O33" s="7" t="inlineStr">
+        <is>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr"/>
@@ -2498,25 +2498,25 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>718981</t>
+          <t>796410</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>65101</v>
+        <v>273361</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>7590002023228</t>
+          <t>7500435153072</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>VICK XPE 44E 120ML</t>
+          <t>VICK XPE INFANTIL 120ML</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>XAROPE 44 E 1,30+13,30MG/ML XPE FR 120ML</t>
+          <t>XAROPE VICK 13,3MG/ML XPE FR 120ML</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
@@ -2539,95 +2539,35 @@
         <v>30</v>
       </c>
       <c r="L34" s="4" t="n">
-        <v>30.73</v>
+        <v>28.7378571428571</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>23.2152</v>
+        <v>24.3825</v>
       </c>
       <c r="N34" s="5">
         <f>K34/L34-1</f>
         <v/>
       </c>
-      <c r="O34" s="7" t="inlineStr">
-        <is>
-          <t>OK (≤ últ. compra)</t>
+      <c r="O34" s="6" t="inlineStr">
+        <is>
+          <t>ACIMA +4.4% (vs últ. compra)</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>796410</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>273361</v>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>7500435153072</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>VICK XPE INFANTIL 120ML</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>XAROPE VICK 13,3MG/ML XPE FR 120ML</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="H35" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="I35" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="J35" s="4">
-        <f>G35*I35</f>
-        <v/>
-      </c>
-      <c r="K35" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="L35" s="4" t="n">
-        <v>28.7378571428571</v>
-      </c>
-      <c r="M35" s="4" t="n">
-        <v>24.3825</v>
-      </c>
-      <c r="N35" s="5">
-        <f>K35/L35-1</f>
-        <v/>
-      </c>
-      <c r="O35" s="6" t="inlineStr">
-        <is>
-          <t>ACIMA +4.4% (vs últ. compra)</t>
-        </is>
-      </c>
-      <c r="P35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="J36" s="9">
-        <f>SUM(J2:J35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="10" t="inlineStr">
+      <c r="J35" s="9">
+        <f>SUM(J2:J34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>Preços da cotação SB LOG de 04/09/2026. 'Menor hist. (un)' = menor entre melhores 3/6/12 meses; 'Últ. compra (un)' = compra atual. Status OK quando o preço unit. equivalente é ≤ menor histórico ou ≤ última compra. 'Qtd pedido' na base de faturamento do distribuidor (caixa ou unidade); 'Un. totais' = unidades da lista de compra.</t>
         </is>

</xml_diff>